<commit_message>
Adição da primeira versão do Frontend. Bugs surgiram no backend no cálculo das comissões por recebimento e na reconciliação
</commit_message>
<xml_diff>
--- a/Conversões.xlsx
+++ b/Conversões.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="30">
   <si>
     <t>Código Produto</t>
   </si>
@@ -22,9 +22,6 @@
     <t>Descrição Produto</t>
   </si>
   <si>
-    <t>Qtde Atendida</t>
-  </si>
-  <si>
     <t>Operação</t>
   </si>
   <si>
@@ -52,21 +49,9 @@
     <t>Gerente Comercial-Pedido</t>
   </si>
   <si>
-    <t>Aplicação Mat./Serv.</t>
-  </si>
-  <si>
     <t>Cliente</t>
   </si>
   <si>
-    <t>Nome Cliente</t>
-  </si>
-  <si>
-    <t>Cidade</t>
-  </si>
-  <si>
-    <t>UF</t>
-  </si>
-  <si>
     <t>Tipo de Mercadoria</t>
   </si>
   <si>
@@ -79,28 +64,13 @@
     <t>Negócio</t>
   </si>
   <si>
-    <t>YSI103740Y</t>
-  </si>
-  <si>
-    <t>YSI109813Y</t>
-  </si>
-  <si>
-    <t>YSI1FD560Y</t>
-  </si>
-  <si>
-    <t>SENSOR YSI IDS COMBINADO DE PH E TEMPERATURA - CABO DE 1,5 METROS</t>
-  </si>
-  <si>
-    <t>SUPORTE PARA SENSORES IDS PARA INSTRUMENTOS YSI MULTILAB</t>
-  </si>
-  <si>
-    <t>ANALISADOR DE BANCADA YSI MULTILAB IDS (DUPLO CANAL)</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>PVEN - PEDIDO DE VENDA</t>
+    <t>QED-AP4-RET</t>
+  </si>
+  <si>
+    <t>Teste Retenção (Neimar)</t>
+  </si>
+  <si>
+    <t>PVEN</t>
   </si>
   <si>
     <t>999999</t>
@@ -112,49 +82,28 @@
     <t>100</t>
   </si>
   <si>
-    <t>SAMANTA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KELLY AMARAL BISPO                      </t>
-  </si>
-  <si>
-    <t>HIDROLOGIA</t>
-  </si>
-  <si>
-    <t>8648</t>
-  </si>
-  <si>
-    <t>BRK AMBIENTAL - RIO CLARO S.A.</t>
-  </si>
-  <si>
-    <t>RIO CLARO</t>
-  </si>
-  <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>Reposição</t>
+    <t>DENER.MARTINS</t>
+  </si>
+  <si>
+    <t>Cliente Teste1</t>
+  </si>
+  <si>
+    <t>Cliente Teste2</t>
+  </si>
+  <si>
+    <t>Cliente Teste3</t>
   </si>
   <si>
     <t>Produto</t>
   </si>
   <si>
-    <t>Sensor</t>
-  </si>
-  <si>
-    <t>Acessório</t>
-  </si>
-  <si>
-    <t>MULTILAB</t>
-  </si>
-  <si>
-    <t>Sonda Portátil</t>
-  </si>
-  <si>
-    <t>Sonda Serie MultiLab</t>
-  </si>
-  <si>
-    <t>Hidrologia</t>
+    <t>Auto Pump</t>
+  </si>
+  <si>
+    <t>Elevador de Liquidos Fixo</t>
+  </si>
+  <si>
+    <t>Remediação</t>
   </si>
 </sst>
 </file>
@@ -516,10 +465,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:21">
+    <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -568,206 +517,269 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:16">
+      <c r="A2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="B2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="C2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="D2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="E2" t="s">
         <v>20</v>
       </c>
+      <c r="F2" s="2">
+        <v>45918</v>
+      </c>
+      <c r="G2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P2" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="2" spans="1:21">
-      <c r="A2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="3" spans="1:16">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="2">
+        <v>45918</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3" t="s">
         <v>24</v>
       </c>
-      <c r="C2" t="s">
+      <c r="M3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N3" t="s">
         <v>27</v>
       </c>
-      <c r="D2" t="s">
+      <c r="O3" t="s">
         <v>28</v>
       </c>
-      <c r="E2" t="s">
+      <c r="P3" t="s">
         <v>29</v>
       </c>
-      <c r="F2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G2" s="2">
-        <v>45880</v>
-      </c>
-      <c r="H2" t="s">
-        <v>31</v>
-      </c>
-      <c r="I2" t="s">
-        <v>31</v>
-      </c>
-      <c r="J2" t="s">
-        <v>32</v>
-      </c>
-      <c r="K2" t="s">
-        <v>33</v>
-      </c>
-      <c r="M2" t="s">
-        <v>34</v>
-      </c>
-      <c r="N2" t="s">
-        <v>35</v>
-      </c>
-      <c r="O2" t="s">
-        <v>36</v>
-      </c>
-      <c r="P2" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R2" t="s">
-        <v>39</v>
-      </c>
-      <c r="S2" t="s">
-        <v>41</v>
-      </c>
-      <c r="T2" t="s">
-        <v>44</v>
-      </c>
-      <c r="U2" t="s">
-        <v>46</v>
-      </c>
     </row>
-    <row r="3" spans="1:21">
-      <c r="A3" t="s">
+    <row r="4" spans="1:16">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="2">
+        <v>45918</v>
+      </c>
+      <c r="G4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" t="s">
         <v>22</v>
       </c>
-      <c r="B3" t="s">
+      <c r="L4" t="s">
         <v>25</v>
       </c>
-      <c r="C3" t="s">
+      <c r="M4" t="s">
+        <v>26</v>
+      </c>
+      <c r="N4" t="s">
         <v>27</v>
       </c>
-      <c r="D3" t="s">
+      <c r="O4" t="s">
         <v>28</v>
       </c>
-      <c r="E3" t="s">
+      <c r="P4" t="s">
         <v>29</v>
       </c>
-      <c r="F3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" s="2">
-        <v>45880</v>
-      </c>
-      <c r="H3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I3" t="s">
-        <v>31</v>
-      </c>
-      <c r="J3" t="s">
-        <v>32</v>
-      </c>
-      <c r="K3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M3" t="s">
-        <v>34</v>
-      </c>
-      <c r="N3" t="s">
-        <v>35</v>
-      </c>
-      <c r="O3" t="s">
-        <v>36</v>
-      </c>
-      <c r="P3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>38</v>
-      </c>
-      <c r="R3" t="s">
-        <v>39</v>
-      </c>
-      <c r="S3" t="s">
-        <v>42</v>
-      </c>
-      <c r="T3" t="s">
-        <v>44</v>
-      </c>
-      <c r="U3" t="s">
-        <v>46</v>
-      </c>
     </row>
-    <row r="4" spans="1:21">
-      <c r="A4" t="s">
+    <row r="5" spans="1:16">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="2">
+        <v>45918</v>
+      </c>
+      <c r="G5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L5" t="s">
         <v>23</v>
       </c>
-      <c r="B4" t="s">
+      <c r="M5" t="s">
         <v>26</v>
       </c>
-      <c r="C4" t="s">
+      <c r="N5" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
+      <c r="O5" t="s">
         <v>28</v>
       </c>
-      <c r="E4" t="s">
+      <c r="P5" t="s">
         <v>29</v>
       </c>
-      <c r="F4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G4" s="2">
-        <v>45880</v>
-      </c>
-      <c r="H4" t="s">
-        <v>31</v>
-      </c>
-      <c r="I4" t="s">
-        <v>31</v>
-      </c>
-      <c r="J4" t="s">
-        <v>32</v>
-      </c>
-      <c r="K4" t="s">
-        <v>33</v>
-      </c>
-      <c r="M4" t="s">
-        <v>34</v>
-      </c>
-      <c r="N4" t="s">
-        <v>35</v>
-      </c>
-      <c r="O4" t="s">
-        <v>36</v>
-      </c>
-      <c r="P4" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>38</v>
-      </c>
-      <c r="R4" t="s">
-        <v>40</v>
-      </c>
-      <c r="S4" t="s">
-        <v>43</v>
-      </c>
-      <c r="T4" t="s">
-        <v>45</v>
-      </c>
-      <c r="U4" t="s">
-        <v>46</v>
+    </row>
+    <row r="6" spans="1:16">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="2">
+        <v>45918</v>
+      </c>
+      <c r="G6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" t="s">
+        <v>22</v>
+      </c>
+      <c r="L6" t="s">
+        <v>24</v>
+      </c>
+      <c r="M6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O6" t="s">
+        <v>28</v>
+      </c>
+      <c r="P6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="2">
+        <v>45918</v>
+      </c>
+      <c r="G7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N7" t="s">
+        <v>27</v>
+      </c>
+      <c r="O7" t="s">
+        <v>28</v>
+      </c>
+      <c r="P7" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rollback para snapshot de <HASH_DO_COMMIT>
</commit_message>
<xml_diff>
--- a/Conversões.xlsx
+++ b/Conversões.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="47">
   <si>
     <t>Código Produto</t>
   </si>
@@ -22,6 +22,9 @@
     <t>Descrição Produto</t>
   </si>
   <si>
+    <t>Qtde Atendida</t>
+  </si>
+  <si>
     <t>Operação</t>
   </si>
   <si>
@@ -49,9 +52,21 @@
     <t>Gerente Comercial-Pedido</t>
   </si>
   <si>
+    <t>Aplicação Mat./Serv.</t>
+  </si>
+  <si>
     <t>Cliente</t>
   </si>
   <si>
+    <t>Nome Cliente</t>
+  </si>
+  <si>
+    <t>Cidade</t>
+  </si>
+  <si>
+    <t>UF</t>
+  </si>
+  <si>
     <t>Tipo de Mercadoria</t>
   </si>
   <si>
@@ -64,13 +79,28 @@
     <t>Negócio</t>
   </si>
   <si>
-    <t>QED-AP4-RET</t>
-  </si>
-  <si>
-    <t>Teste Retenção (Neimar)</t>
-  </si>
-  <si>
-    <t>PVEN</t>
+    <t>YSI103740Y</t>
+  </si>
+  <si>
+    <t>YSI109813Y</t>
+  </si>
+  <si>
+    <t>YSI1FD560Y</t>
+  </si>
+  <si>
+    <t>SENSOR YSI IDS COMBINADO DE PH E TEMPERATURA - CABO DE 1,5 METROS</t>
+  </si>
+  <si>
+    <t>SUPORTE PARA SENSORES IDS PARA INSTRUMENTOS YSI MULTILAB</t>
+  </si>
+  <si>
+    <t>ANALISADOR DE BANCADA YSI MULTILAB IDS (DUPLO CANAL)</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>PVEN - PEDIDO DE VENDA</t>
   </si>
   <si>
     <t>999999</t>
@@ -82,28 +112,49 @@
     <t>100</t>
   </si>
   <si>
-    <t>DENER.MARTINS</t>
-  </si>
-  <si>
-    <t>Cliente Teste1</t>
-  </si>
-  <si>
-    <t>Cliente Teste2</t>
-  </si>
-  <si>
-    <t>Cliente Teste3</t>
+    <t>SAMANTA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KELLY AMARAL BISPO                      </t>
+  </si>
+  <si>
+    <t>HIDROLOGIA</t>
+  </si>
+  <si>
+    <t>8648</t>
+  </si>
+  <si>
+    <t>BRK AMBIENTAL - RIO CLARO S.A.</t>
+  </si>
+  <si>
+    <t>RIO CLARO</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>Reposição</t>
   </si>
   <si>
     <t>Produto</t>
   </si>
   <si>
-    <t>Auto Pump</t>
-  </si>
-  <si>
-    <t>Elevador de Liquidos Fixo</t>
-  </si>
-  <si>
-    <t>Remediação</t>
+    <t>Sensor</t>
+  </si>
+  <si>
+    <t>Acessório</t>
+  </si>
+  <si>
+    <t>MULTILAB</t>
+  </si>
+  <si>
+    <t>Sonda Portátil</t>
+  </si>
+  <si>
+    <t>Sonda Serie MultiLab</t>
+  </si>
+  <si>
+    <t>Hidrologia</t>
   </si>
 </sst>
 </file>
@@ -465,10 +516,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:21">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -517,269 +568,206 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:21">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="2">
-        <v>45918</v>
-      </c>
-      <c r="G2" t="s">
-        <v>21</v>
+        <v>29</v>
+      </c>
+      <c r="F2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="2">
+        <v>45880</v>
       </c>
       <c r="H2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="I2" t="s">
+        <v>31</v>
+      </c>
+      <c r="J2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N2" t="s">
+        <v>35</v>
+      </c>
+      <c r="O2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P2" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R2" t="s">
+        <v>39</v>
+      </c>
+      <c r="S2" t="s">
+        <v>41</v>
+      </c>
+      <c r="T2" t="s">
+        <v>44</v>
+      </c>
+      <c r="U2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21">
+      <c r="A3" t="s">
         <v>22</v>
       </c>
-      <c r="L2" t="s">
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" s="2">
+        <v>45880</v>
+      </c>
+      <c r="H3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I3" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N3" t="s">
+        <v>35</v>
+      </c>
+      <c r="O3" t="s">
+        <v>36</v>
+      </c>
+      <c r="P3" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>38</v>
+      </c>
+      <c r="R3" t="s">
+        <v>39</v>
+      </c>
+      <c r="S3" t="s">
+        <v>42</v>
+      </c>
+      <c r="T3" t="s">
+        <v>44</v>
+      </c>
+      <c r="U3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21">
+      <c r="A4" t="s">
         <v>23</v>
       </c>
-      <c r="M2" t="s">
+      <c r="B4" t="s">
         <v>26</v>
       </c>
-      <c r="N2" t="s">
+      <c r="C4" t="s">
         <v>27</v>
       </c>
-      <c r="O2" t="s">
+      <c r="D4" t="s">
         <v>28</v>
       </c>
-      <c r="P2" t="s">
+      <c r="E4" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="3" spans="1:16">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" s="2">
-        <v>45918</v>
-      </c>
-      <c r="G3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I3" t="s">
-        <v>22</v>
-      </c>
-      <c r="L3" t="s">
-        <v>24</v>
-      </c>
-      <c r="M3" t="s">
-        <v>26</v>
-      </c>
-      <c r="N3" t="s">
-        <v>27</v>
-      </c>
-      <c r="O3" t="s">
-        <v>28</v>
-      </c>
-      <c r="P3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="2">
-        <v>45918</v>
-      </c>
-      <c r="G4" t="s">
-        <v>21</v>
+      <c r="F4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="2">
+        <v>45880</v>
       </c>
       <c r="H4" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="I4" t="s">
-        <v>22</v>
-      </c>
-      <c r="L4" t="s">
-        <v>25</v>
+        <v>31</v>
+      </c>
+      <c r="J4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K4" t="s">
+        <v>33</v>
       </c>
       <c r="M4" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="N4" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="O4" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="P4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="2">
-        <v>45918</v>
-      </c>
-      <c r="G5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" t="s">
-        <v>22</v>
-      </c>
-      <c r="L5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M5" t="s">
-        <v>26</v>
-      </c>
-      <c r="N5" t="s">
-        <v>27</v>
-      </c>
-      <c r="O5" t="s">
-        <v>28</v>
-      </c>
-      <c r="P5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16">
-      <c r="A6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="2">
-        <v>45918</v>
-      </c>
-      <c r="G6" t="s">
-        <v>21</v>
-      </c>
-      <c r="H6" t="s">
-        <v>21</v>
-      </c>
-      <c r="I6" t="s">
-        <v>22</v>
-      </c>
-      <c r="L6" t="s">
-        <v>24</v>
-      </c>
-      <c r="M6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N6" t="s">
-        <v>27</v>
-      </c>
-      <c r="O6" t="s">
-        <v>28</v>
-      </c>
-      <c r="P6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16">
-      <c r="A7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" s="2">
-        <v>45918</v>
-      </c>
-      <c r="G7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7" t="s">
-        <v>21</v>
-      </c>
-      <c r="I7" t="s">
-        <v>22</v>
-      </c>
-      <c r="L7" t="s">
-        <v>23</v>
-      </c>
-      <c r="M7" t="s">
-        <v>26</v>
-      </c>
-      <c r="N7" t="s">
-        <v>27</v>
-      </c>
-      <c r="O7" t="s">
-        <v>28</v>
-      </c>
-      <c r="P7" t="s">
-        <v>29</v>
+        <v>37</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>38</v>
+      </c>
+      <c r="R4" t="s">
+        <v>40</v>
+      </c>
+      <c r="S4" t="s">
+        <v>43</v>
+      </c>
+      <c r="T4" t="s">
+        <v>45</v>
+      </c>
+      <c r="U4" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BACKEND FUNCIONAL COM GERAÇÃO CORRETA DOS ARQUIVOS - VERSÃO 1.0
</commit_message>
<xml_diff>
--- a/Conversões.xlsx
+++ b/Conversões.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="51">
   <si>
     <t>Código Produto</t>
   </si>
@@ -79,31 +79,46 @@
     <t>Negócio</t>
   </si>
   <si>
-    <t>YSI103740Y</t>
-  </si>
-  <si>
-    <t>YSI109813Y</t>
-  </si>
-  <si>
-    <t>YSI1FD560Y</t>
-  </si>
-  <si>
-    <t>SENSOR YSI IDS COMBINADO DE PH E TEMPERATURA - CABO DE 1,5 METROS</t>
-  </si>
-  <si>
-    <t>SUPORTE PARA SENSORES IDS PARA INSTRUMENTOS YSI MULTILAB</t>
-  </si>
-  <si>
-    <t>ANALISADOR DE BANCADA YSI MULTILAB IDS (DUPLO CANAL)</t>
+    <t>HONMMS-G2</t>
+  </si>
+  <si>
+    <t>HONMMS-TR</t>
+  </si>
+  <si>
+    <t>HONMMS-D2</t>
+  </si>
+  <si>
+    <t>ANGLTA2051WJ24V-IND</t>
+  </si>
+  <si>
+    <t>HONMMT-01</t>
+  </si>
+  <si>
+    <t>SENSOR ELETROQUIMICO DE H2 PARA ANALISADOR DE GÁS MODELO MIDAS M</t>
+  </si>
+  <si>
+    <t>SENSOR IR DE CO2 PARA ANALISADOR DE GÁS MODELO MIDAS M</t>
+  </si>
+  <si>
+    <t>SENSOR DE OXIGÊNIO PARA USO NO ANALISADOR DE GASES MODELO MIDAS M</t>
+  </si>
+  <si>
+    <t>SIRENE P/ SISTEMA DE DETECÇÃO FIXA SAV-C 24V</t>
+  </si>
+  <si>
+    <t>ANALISADOR FIXO PARA 4 GASES - MODELO MIDAS M</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
+    <t>2</t>
+  </si>
+  <si>
     <t>PVEN - PEDIDO DE VENDA</t>
   </si>
   <si>
-    <t>999999</t>
+    <t>133701</t>
   </si>
   <si>
     <t>FATURADO</t>
@@ -112,22 +127,22 @@
     <t>100</t>
   </si>
   <si>
-    <t>SAMANTA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KELLY AMARAL BISPO                      </t>
-  </si>
-  <si>
-    <t>HIDROLOGIA</t>
-  </si>
-  <si>
-    <t>8648</t>
-  </si>
-  <si>
-    <t>BRK AMBIENTAL - RIO CLARO S.A.</t>
-  </si>
-  <si>
-    <t>RIO CLARO</t>
+    <t>ANDREY.ANDRADE</t>
+  </si>
+  <si>
+    <t>LEONARDO DO CARMO</t>
+  </si>
+  <si>
+    <t>DEPART. DETECÇÃO FIXA GASES</t>
+  </si>
+  <si>
+    <t>22853</t>
+  </si>
+  <si>
+    <t>AMYRIS FERMENTACAO DE PERFORMANCE LTDA</t>
+  </si>
+  <si>
+    <t>BARRA BONITA</t>
   </si>
   <si>
     <t>SP</t>
@@ -145,16 +160,13 @@
     <t>Acessório</t>
   </si>
   <si>
-    <t>MULTILAB</t>
-  </si>
-  <si>
-    <t>Sonda Portátil</t>
-  </si>
-  <si>
-    <t>Sonda Serie MultiLab</t>
-  </si>
-  <si>
-    <t>Hidrologia</t>
+    <t>Midas</t>
+  </si>
+  <si>
+    <t>Detector Fixo</t>
+  </si>
+  <si>
+    <t>SSO</t>
   </si>
 </sst>
 </file>
@@ -516,7 +528,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:21">
@@ -589,61 +601,64 @@
         <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="G2" s="2">
-        <v>45880</v>
+        <v>45904</v>
       </c>
       <c r="H2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="I2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="J2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="K2" t="s">
-        <v>33</v>
+        <v>38</v>
+      </c>
+      <c r="L2" t="s">
+        <v>38</v>
       </c>
       <c r="M2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="N2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="O2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="Q2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="R2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="S2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="T2" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="U2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -651,61 +666,64 @@
         <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E3" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F3" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="G3" s="2">
-        <v>45880</v>
+        <v>45904</v>
       </c>
       <c r="H3" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="I3" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="J3" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="K3" t="s">
-        <v>33</v>
+        <v>38</v>
+      </c>
+      <c r="L3" t="s">
+        <v>38</v>
       </c>
       <c r="M3" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="N3" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="O3" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P3" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="Q3" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="R3" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="S3" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="T3" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="U3" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -713,61 +731,194 @@
         <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" s="2">
+        <v>45904</v>
+      </c>
+      <c r="H4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" t="s">
+        <v>37</v>
+      </c>
+      <c r="K4" t="s">
+        <v>38</v>
+      </c>
+      <c r="L4" t="s">
+        <v>38</v>
+      </c>
+      <c r="M4" t="s">
+        <v>39</v>
+      </c>
+      <c r="N4" t="s">
+        <v>40</v>
+      </c>
+      <c r="O4" t="s">
+        <v>41</v>
+      </c>
+      <c r="P4" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>43</v>
+      </c>
+      <c r="R4" t="s">
+        <v>44</v>
+      </c>
+      <c r="S4" t="s">
+        <v>46</v>
+      </c>
+      <c r="T4" t="s">
+        <v>49</v>
+      </c>
+      <c r="U4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
         <v>29</v>
       </c>
-      <c r="F4" t="s">
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" s="2">
+        <v>45904</v>
+      </c>
+      <c r="H5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J5" t="s">
+        <v>37</v>
+      </c>
+      <c r="K5" t="s">
+        <v>38</v>
+      </c>
+      <c r="L5" t="s">
+        <v>38</v>
+      </c>
+      <c r="M5" t="s">
+        <v>39</v>
+      </c>
+      <c r="N5" t="s">
+        <v>40</v>
+      </c>
+      <c r="O5" t="s">
+        <v>41</v>
+      </c>
+      <c r="P5" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>43</v>
+      </c>
+      <c r="R5" t="s">
+        <v>45</v>
+      </c>
+      <c r="S5" t="s">
+        <v>47</v>
+      </c>
+      <c r="T5" t="s">
+        <v>49</v>
+      </c>
+      <c r="U5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="2">
-        <v>45880</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="C6" t="s">
         <v>31</v>
       </c>
-      <c r="I4" t="s">
-        <v>31</v>
-      </c>
-      <c r="J4" t="s">
-        <v>32</v>
-      </c>
-      <c r="K4" t="s">
+      <c r="D6" t="s">
         <v>33</v>
       </c>
-      <c r="M4" t="s">
+      <c r="E6" t="s">
         <v>34</v>
       </c>
-      <c r="N4" t="s">
+      <c r="F6" t="s">
         <v>35</v>
       </c>
-      <c r="O4" t="s">
+      <c r="G6" s="2">
+        <v>45904</v>
+      </c>
+      <c r="H6" t="s">
         <v>36</v>
       </c>
-      <c r="P4" t="s">
+      <c r="I6" t="s">
+        <v>36</v>
+      </c>
+      <c r="J6" t="s">
         <v>37</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="K6" t="s">
         <v>38</v>
       </c>
-      <c r="R4" t="s">
+      <c r="L6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M6" t="s">
+        <v>39</v>
+      </c>
+      <c r="N6" t="s">
         <v>40</v>
       </c>
-      <c r="S4" t="s">
+      <c r="O6" t="s">
+        <v>41</v>
+      </c>
+      <c r="P6" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q6" t="s">
         <v>43</v>
       </c>
-      <c r="T4" t="s">
+      <c r="R6" t="s">
         <v>45</v>
       </c>
-      <c r="U4" t="s">
-        <v>46</v>
+      <c r="S6" t="s">
+        <v>48</v>
+      </c>
+      <c r="T6" t="s">
+        <v>49</v>
+      </c>
+      <c r="U6" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>